<commit_message>
Fix: license prefix, client address, section order, form reset
</commit_message>
<xml_diff>
--- a/Template ADU.xlsx
+++ b/Template ADU.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\camek\OneDrive\Рабочий стол\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\camek\estimator-pro\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AEE7A97-95DE-4FCA-A595-986FE8589D99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1515" yWindow="960" windowWidth="32970" windowHeight="19920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template 6.0 (FHR and other PCA" sheetId="1" r:id="rId1"/>
@@ -19771,8 +19771,6 @@
     <mergeCell ref="E943:E944"/>
     <mergeCell ref="D933:D934"/>
     <mergeCell ref="E933:E934"/>
-    <mergeCell ref="B933:B934"/>
-    <mergeCell ref="C933:C934"/>
     <mergeCell ref="D902:D903"/>
     <mergeCell ref="E902:E903"/>
     <mergeCell ref="C904:C905"/>
@@ -19824,6 +19822,8 @@
     <mergeCell ref="E939:E940"/>
     <mergeCell ref="B941:B942"/>
     <mergeCell ref="C941:C942"/>
+    <mergeCell ref="B933:B934"/>
+    <mergeCell ref="C933:C934"/>
     <mergeCell ref="D957:D958"/>
     <mergeCell ref="E957:E958"/>
     <mergeCell ref="F943:F944"/>
@@ -19842,6 +19842,14 @@
     <mergeCell ref="C967:C968"/>
     <mergeCell ref="D967:D968"/>
     <mergeCell ref="E967:E968"/>
+    <mergeCell ref="E965:E966"/>
+    <mergeCell ref="B961:B962"/>
+    <mergeCell ref="B963:B964"/>
+    <mergeCell ref="C963:C964"/>
+    <mergeCell ref="D963:D964"/>
+    <mergeCell ref="E963:E964"/>
+    <mergeCell ref="B965:B966"/>
+    <mergeCell ref="C965:C966"/>
     <mergeCell ref="C969:C970"/>
     <mergeCell ref="D969:D970"/>
     <mergeCell ref="E969:E970"/>
@@ -19874,14 +19882,6 @@
     <mergeCell ref="D961:D962"/>
     <mergeCell ref="E961:E962"/>
     <mergeCell ref="D965:D966"/>
-    <mergeCell ref="E965:E966"/>
-    <mergeCell ref="B961:B962"/>
-    <mergeCell ref="B963:B964"/>
-    <mergeCell ref="C963:C964"/>
-    <mergeCell ref="D963:D964"/>
-    <mergeCell ref="E963:E964"/>
-    <mergeCell ref="B965:B966"/>
-    <mergeCell ref="C965:C966"/>
     <mergeCell ref="D973:D974"/>
     <mergeCell ref="E973:E974"/>
     <mergeCell ref="D981:D982"/>
@@ -19902,13 +19902,18 @@
     <mergeCell ref="C156:C157"/>
     <mergeCell ref="D156:D157"/>
     <mergeCell ref="E156:E157"/>
-    <mergeCell ref="F114:F115"/>
-    <mergeCell ref="C116:C117"/>
-    <mergeCell ref="F116:F117"/>
-    <mergeCell ref="B116:B117"/>
-    <mergeCell ref="B118:B119"/>
-    <mergeCell ref="C118:C119"/>
-    <mergeCell ref="D118:D119"/>
+    <mergeCell ref="C164:C165"/>
+    <mergeCell ref="D164:D165"/>
+    <mergeCell ref="E164:E165"/>
+    <mergeCell ref="C166:C167"/>
+    <mergeCell ref="D166:D167"/>
+    <mergeCell ref="E166:E167"/>
+    <mergeCell ref="B166:B167"/>
+    <mergeCell ref="B168:B169"/>
+    <mergeCell ref="C168:C169"/>
+    <mergeCell ref="D168:D169"/>
+    <mergeCell ref="E168:E169"/>
+    <mergeCell ref="B170:B171"/>
     <mergeCell ref="E118:E119"/>
     <mergeCell ref="B120:B121"/>
     <mergeCell ref="C120:C121"/>
@@ -19934,8 +19939,6 @@
     <mergeCell ref="E116:E117"/>
     <mergeCell ref="D120:D121"/>
     <mergeCell ref="E120:E121"/>
-    <mergeCell ref="F120:F121"/>
-    <mergeCell ref="B126:B127"/>
     <mergeCell ref="B128:B129"/>
     <mergeCell ref="C128:C129"/>
     <mergeCell ref="D128:D129"/>
@@ -19966,6 +19969,8 @@
     <mergeCell ref="D16:D17"/>
     <mergeCell ref="E16:E17"/>
     <mergeCell ref="F16:F17"/>
+    <mergeCell ref="F114:F115"/>
+    <mergeCell ref="C116:C117"/>
     <mergeCell ref="A18:E18"/>
     <mergeCell ref="A19:D19"/>
     <mergeCell ref="D22:D23"/>
@@ -20072,6 +20077,19 @@
     <mergeCell ref="C72:C73"/>
     <mergeCell ref="D72:D73"/>
     <mergeCell ref="E72:E73"/>
+    <mergeCell ref="E94:E95"/>
+    <mergeCell ref="F94:F95"/>
+    <mergeCell ref="B92:B93"/>
+    <mergeCell ref="C92:C93"/>
+    <mergeCell ref="D92:D93"/>
+    <mergeCell ref="E92:E93"/>
+    <mergeCell ref="B94:B95"/>
+    <mergeCell ref="C94:C95"/>
+    <mergeCell ref="D94:D95"/>
+    <mergeCell ref="A96:E96"/>
+    <mergeCell ref="A97:D97"/>
+    <mergeCell ref="B98:B99"/>
+    <mergeCell ref="C98:C99"/>
     <mergeCell ref="F72:F75"/>
     <mergeCell ref="B74:B75"/>
     <mergeCell ref="C74:C75"/>
@@ -20090,7 +20108,6 @@
     <mergeCell ref="D82:D83"/>
     <mergeCell ref="E82:E83"/>
     <mergeCell ref="F82:F83"/>
-    <mergeCell ref="E104:E105"/>
     <mergeCell ref="E86:E87"/>
     <mergeCell ref="F86:F87"/>
     <mergeCell ref="F88:F91"/>
@@ -20109,19 +20126,6 @@
     <mergeCell ref="B90:B91"/>
     <mergeCell ref="C90:C91"/>
     <mergeCell ref="D90:D91"/>
-    <mergeCell ref="E94:E95"/>
-    <mergeCell ref="F94:F95"/>
-    <mergeCell ref="B92:B93"/>
-    <mergeCell ref="C92:C93"/>
-    <mergeCell ref="D92:D93"/>
-    <mergeCell ref="E92:E93"/>
-    <mergeCell ref="B94:B95"/>
-    <mergeCell ref="C94:C95"/>
-    <mergeCell ref="D94:D95"/>
-    <mergeCell ref="A96:E96"/>
-    <mergeCell ref="A97:D97"/>
-    <mergeCell ref="B98:B99"/>
-    <mergeCell ref="C98:C99"/>
     <mergeCell ref="D98:D99"/>
     <mergeCell ref="E98:E99"/>
     <mergeCell ref="B100:B101"/>
@@ -20146,13 +20150,14 @@
     <mergeCell ref="C102:C103"/>
     <mergeCell ref="D102:D103"/>
     <mergeCell ref="E102:E103"/>
-    <mergeCell ref="C164:C165"/>
-    <mergeCell ref="D164:D165"/>
-    <mergeCell ref="E164:E165"/>
-    <mergeCell ref="C166:C167"/>
-    <mergeCell ref="D166:D167"/>
-    <mergeCell ref="E166:E167"/>
-    <mergeCell ref="B166:B167"/>
+    <mergeCell ref="E104:E105"/>
+    <mergeCell ref="F120:F121"/>
+    <mergeCell ref="B126:B127"/>
+    <mergeCell ref="F116:F117"/>
+    <mergeCell ref="B116:B117"/>
+    <mergeCell ref="B118:B119"/>
+    <mergeCell ref="C118:C119"/>
+    <mergeCell ref="D118:D119"/>
     <mergeCell ref="F132:F133"/>
     <mergeCell ref="E136:E137"/>
     <mergeCell ref="F136:F137"/>
@@ -20172,11 +20177,6 @@
     <mergeCell ref="B140:B141"/>
     <mergeCell ref="C140:C141"/>
     <mergeCell ref="D140:D141"/>
-    <mergeCell ref="B168:B169"/>
-    <mergeCell ref="C168:C169"/>
-    <mergeCell ref="D168:D169"/>
-    <mergeCell ref="E168:E169"/>
-    <mergeCell ref="B170:B171"/>
     <mergeCell ref="C170:C171"/>
     <mergeCell ref="E174:E175"/>
     <mergeCell ref="F174:F175"/>
@@ -20256,6 +20256,10 @@
     <mergeCell ref="D188:D189"/>
     <mergeCell ref="E188:E189"/>
     <mergeCell ref="B190:B191"/>
+    <mergeCell ref="C190:C191"/>
+    <mergeCell ref="B192:B193"/>
+    <mergeCell ref="C192:C193"/>
+    <mergeCell ref="D192:D193"/>
     <mergeCell ref="F210:F211"/>
     <mergeCell ref="A212:D212"/>
     <mergeCell ref="D204:D205"/>
@@ -20288,10 +20292,6 @@
     <mergeCell ref="E182:E183"/>
     <mergeCell ref="C200:C201"/>
     <mergeCell ref="D200:D201"/>
-    <mergeCell ref="C190:C191"/>
-    <mergeCell ref="B192:B193"/>
-    <mergeCell ref="C192:C193"/>
-    <mergeCell ref="D192:D193"/>
     <mergeCell ref="E192:E193"/>
     <mergeCell ref="A194:E194"/>
     <mergeCell ref="A195:D195"/>
@@ -36095,8 +36095,6 @@
     <mergeCell ref="E943:E944"/>
     <mergeCell ref="D933:D934"/>
     <mergeCell ref="E933:E934"/>
-    <mergeCell ref="B933:B934"/>
-    <mergeCell ref="C933:C934"/>
     <mergeCell ref="D902:D903"/>
     <mergeCell ref="E902:E903"/>
     <mergeCell ref="C904:C905"/>
@@ -36148,6 +36146,8 @@
     <mergeCell ref="E939:E940"/>
     <mergeCell ref="B941:B942"/>
     <mergeCell ref="C941:C942"/>
+    <mergeCell ref="B933:B934"/>
+    <mergeCell ref="C933:C934"/>
     <mergeCell ref="D957:D958"/>
     <mergeCell ref="E957:E958"/>
     <mergeCell ref="F943:F944"/>
@@ -36166,6 +36166,14 @@
     <mergeCell ref="C967:C968"/>
     <mergeCell ref="D967:D968"/>
     <mergeCell ref="E967:E968"/>
+    <mergeCell ref="E965:E966"/>
+    <mergeCell ref="B961:B962"/>
+    <mergeCell ref="B963:B964"/>
+    <mergeCell ref="C963:C964"/>
+    <mergeCell ref="D963:D964"/>
+    <mergeCell ref="E963:E964"/>
+    <mergeCell ref="B965:B966"/>
+    <mergeCell ref="C965:C966"/>
     <mergeCell ref="C969:C970"/>
     <mergeCell ref="D969:D970"/>
     <mergeCell ref="E969:E970"/>
@@ -36198,14 +36206,6 @@
     <mergeCell ref="D961:D962"/>
     <mergeCell ref="E961:E962"/>
     <mergeCell ref="D965:D966"/>
-    <mergeCell ref="E965:E966"/>
-    <mergeCell ref="B961:B962"/>
-    <mergeCell ref="B963:B964"/>
-    <mergeCell ref="C963:C964"/>
-    <mergeCell ref="D963:D964"/>
-    <mergeCell ref="E963:E964"/>
-    <mergeCell ref="B965:B966"/>
-    <mergeCell ref="C965:C966"/>
     <mergeCell ref="D973:D974"/>
     <mergeCell ref="E973:E974"/>
     <mergeCell ref="D981:D982"/>
@@ -36226,13 +36226,18 @@
     <mergeCell ref="C156:C157"/>
     <mergeCell ref="D156:D157"/>
     <mergeCell ref="E156:E157"/>
-    <mergeCell ref="F114:F115"/>
-    <mergeCell ref="C116:C117"/>
-    <mergeCell ref="F116:F117"/>
-    <mergeCell ref="B116:B117"/>
-    <mergeCell ref="B118:B119"/>
-    <mergeCell ref="C118:C119"/>
-    <mergeCell ref="D118:D119"/>
+    <mergeCell ref="C164:C165"/>
+    <mergeCell ref="D164:D165"/>
+    <mergeCell ref="E164:E165"/>
+    <mergeCell ref="C166:C167"/>
+    <mergeCell ref="D166:D167"/>
+    <mergeCell ref="E166:E167"/>
+    <mergeCell ref="B166:B167"/>
+    <mergeCell ref="B168:B169"/>
+    <mergeCell ref="C168:C169"/>
+    <mergeCell ref="D168:D169"/>
+    <mergeCell ref="E168:E169"/>
+    <mergeCell ref="B170:B171"/>
     <mergeCell ref="E118:E119"/>
     <mergeCell ref="B120:B121"/>
     <mergeCell ref="C120:C121"/>
@@ -36258,8 +36263,6 @@
     <mergeCell ref="E116:E117"/>
     <mergeCell ref="D120:D121"/>
     <mergeCell ref="E120:E121"/>
-    <mergeCell ref="F120:F121"/>
-    <mergeCell ref="B126:B127"/>
     <mergeCell ref="B128:B129"/>
     <mergeCell ref="C128:C129"/>
     <mergeCell ref="D128:D129"/>
@@ -36290,6 +36293,8 @@
     <mergeCell ref="D16:D17"/>
     <mergeCell ref="E16:E17"/>
     <mergeCell ref="F16:F17"/>
+    <mergeCell ref="F114:F115"/>
+    <mergeCell ref="C116:C117"/>
     <mergeCell ref="A18:E18"/>
     <mergeCell ref="A19:D19"/>
     <mergeCell ref="D22:D23"/>
@@ -36396,6 +36401,19 @@
     <mergeCell ref="C72:C73"/>
     <mergeCell ref="D72:D73"/>
     <mergeCell ref="E72:E73"/>
+    <mergeCell ref="E94:E95"/>
+    <mergeCell ref="F94:F95"/>
+    <mergeCell ref="B92:B93"/>
+    <mergeCell ref="C92:C93"/>
+    <mergeCell ref="D92:D93"/>
+    <mergeCell ref="E92:E93"/>
+    <mergeCell ref="B94:B95"/>
+    <mergeCell ref="C94:C95"/>
+    <mergeCell ref="D94:D95"/>
+    <mergeCell ref="A96:E96"/>
+    <mergeCell ref="A97:D97"/>
+    <mergeCell ref="B98:B99"/>
+    <mergeCell ref="C98:C99"/>
     <mergeCell ref="F72:F75"/>
     <mergeCell ref="B74:B75"/>
     <mergeCell ref="C74:C75"/>
@@ -36414,7 +36432,6 @@
     <mergeCell ref="D82:D83"/>
     <mergeCell ref="E82:E83"/>
     <mergeCell ref="F82:F83"/>
-    <mergeCell ref="E104:E105"/>
     <mergeCell ref="E86:E87"/>
     <mergeCell ref="F86:F87"/>
     <mergeCell ref="F88:F91"/>
@@ -36433,19 +36450,6 @@
     <mergeCell ref="B90:B91"/>
     <mergeCell ref="C90:C91"/>
     <mergeCell ref="D90:D91"/>
-    <mergeCell ref="E94:E95"/>
-    <mergeCell ref="F94:F95"/>
-    <mergeCell ref="B92:B93"/>
-    <mergeCell ref="C92:C93"/>
-    <mergeCell ref="D92:D93"/>
-    <mergeCell ref="E92:E93"/>
-    <mergeCell ref="B94:B95"/>
-    <mergeCell ref="C94:C95"/>
-    <mergeCell ref="D94:D95"/>
-    <mergeCell ref="A96:E96"/>
-    <mergeCell ref="A97:D97"/>
-    <mergeCell ref="B98:B99"/>
-    <mergeCell ref="C98:C99"/>
     <mergeCell ref="D98:D99"/>
     <mergeCell ref="E98:E99"/>
     <mergeCell ref="B100:B101"/>
@@ -36470,13 +36474,14 @@
     <mergeCell ref="C102:C103"/>
     <mergeCell ref="D102:D103"/>
     <mergeCell ref="E102:E103"/>
-    <mergeCell ref="C164:C165"/>
-    <mergeCell ref="D164:D165"/>
-    <mergeCell ref="E164:E165"/>
-    <mergeCell ref="C166:C167"/>
-    <mergeCell ref="D166:D167"/>
-    <mergeCell ref="E166:E167"/>
-    <mergeCell ref="B166:B167"/>
+    <mergeCell ref="E104:E105"/>
+    <mergeCell ref="F120:F121"/>
+    <mergeCell ref="B126:B127"/>
+    <mergeCell ref="F116:F117"/>
+    <mergeCell ref="B116:B117"/>
+    <mergeCell ref="B118:B119"/>
+    <mergeCell ref="C118:C119"/>
+    <mergeCell ref="D118:D119"/>
     <mergeCell ref="F132:F133"/>
     <mergeCell ref="E136:E137"/>
     <mergeCell ref="F136:F137"/>
@@ -36496,11 +36501,6 @@
     <mergeCell ref="B140:B141"/>
     <mergeCell ref="C140:C141"/>
     <mergeCell ref="D140:D141"/>
-    <mergeCell ref="B168:B169"/>
-    <mergeCell ref="C168:C169"/>
-    <mergeCell ref="D168:D169"/>
-    <mergeCell ref="E168:E169"/>
-    <mergeCell ref="B170:B171"/>
     <mergeCell ref="C170:C171"/>
     <mergeCell ref="E174:E175"/>
     <mergeCell ref="F174:F175"/>
@@ -36580,6 +36580,10 @@
     <mergeCell ref="D188:D189"/>
     <mergeCell ref="E188:E189"/>
     <mergeCell ref="B190:B191"/>
+    <mergeCell ref="C190:C191"/>
+    <mergeCell ref="B192:B193"/>
+    <mergeCell ref="C192:C193"/>
+    <mergeCell ref="D192:D193"/>
     <mergeCell ref="F210:F211"/>
     <mergeCell ref="A212:D212"/>
     <mergeCell ref="D204:D205"/>
@@ -36612,10 +36616,6 @@
     <mergeCell ref="E182:E183"/>
     <mergeCell ref="C200:C201"/>
     <mergeCell ref="D200:D201"/>
-    <mergeCell ref="C190:C191"/>
-    <mergeCell ref="B192:B193"/>
-    <mergeCell ref="C192:C193"/>
-    <mergeCell ref="D192:D193"/>
     <mergeCell ref="E192:E193"/>
     <mergeCell ref="A194:E194"/>
     <mergeCell ref="A195:D195"/>

</xml_diff>